<commit_message>
chore: preserve August review worktree source snapshot
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="stories" sheetId="1" state="visible" ns1:id="rId1"/>
+    <sheet name="summary" sheetId="2" state="visible" ns1:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'stories'!$A$1:$U$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'stories'!$A$1:$U$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -612,7 +612,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>解消済み: Android/iPhone物理実機で手動保存、正規化重複通知、既存詳細への復帰を確認。Supabaseはこの端末内保存ストーリーの完了条件ではない。</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-07-03 06:11:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>解消済み: 2026-06-29時点のiPhone共有拡張保存引き継ぎ失敗は、2026-07-02/03の物理iPhone Safari共有再検証で再現せず、保存完了まで確認。CoreSimulator/XCTest不整合は別ゲートとして継続。</t>
+          <t>解消済み: Android ACTION_SENDとiPhone Safari共有拡張で、保存先タグ選択から保存完了・共有元復帰まで物理実機確認済み。Supabase/Store consoleはこの共有受信ストーリーの完了条件ではない。</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-07-03 04:45:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>iPhone physical US-003 input source gap: Safari通常共有は単一URLのみ。Web Share API一時ページでは共有シート生成不可。Notesに2件URL本文を作り、その他アプリ一覧にりんばむは表示されたが、Notes側が共同作業リンク作成フローへ遷移し、Share Extension保存画面まで到達しなかった。 2026-07-03 07:05追加: iPhone実機で追加確認。Notes共有は共有先一覧にりんばむが表示されても、選択後にNotesの「リンクを作成」共同作業UIへ遷移しShare Extensionに渡らない。Safari Web Share検証はCloudflare Quick Tunnelが404、localhost.runがTLS不可。LAN HTTPページは表示できたがSafariで navigator.share is not a function となり、HTTPS入力元なしでは共有シート生成不可。 2026-07-03 07:18追加: HTTPS example.com 上でSafariアドレスバーから javascript:navigator.share(...) を実行する方式も試したが、iPhone Safariが「スクリプトを実行できません。JavaScriptは、この方法で使用することが許されていません。」を表示し共有シートは出なかった。</t>
+          <t>解消済み: 署名済み一時共有元アプリからURLオブジェクト2件をiPhone Share Extensionへ渡し、2件保存完了を物理実機で確認。Android ACTION_SEND_MULTIPLEも物理実機確認済み。</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-07-03 22:48:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>PARTIAL_DEVICE_GAP: Android/iPhone実機で同一URL重複判定は確認。表記違いURLの正規化重複は未検証。iPhone手動追加の重複保存後、コード上は「このURLはすでに保存済みです」+「見る」通知を5秒表示する設計だが、Appium証跡では保存後ホームに戻り通知が見えなかった。</t>
+          <t>解消済み: Android/iPhone物理実機で大文字HTTPS、既定port、fragment差を含む表記違いURLが同一normalizedUrlとして重複扱いになり、重複通知と「見る」導線を確認。</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-07-03 06:16:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>iPhone保存済みURLを用いた絞り込み操作は未検証。Androidでは2026-07-03に自作タグクリックが即解除される不具合を修正済み。</t>
+          <t>解消済み: Android/iPhone物理実機で保存済みデータを用いた自作タグ絞り込みを確認。Supabaseはローカル一覧フィルターの完了条件ではない。</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-07-03 06:16:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>iPhone物理端末での再起動後保持は未検証。AndroidはDataStore保持を実機で確認済み。</t>
+          <t>解消済み: Android/iPhone物理実機で表示モード切替とアプリ再起動後の保持を確認。Supabase/Store consoleはこの端末内設定の完了条件ではない。</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2026-07-03 06:17:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>iPhoneの横スワイプアーカイブ/Undo実行は未検証。Androidは2026-07-03に右スワイプ、Snackbar「元に戻す」、DBのACTIVE復帰まで確認済み。</t>
+          <t>解消済み: Android/iPhone物理実機でActiveカード右スワイプ、アーカイブ通知、Undo、対象のActive復帰を確認。</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>2026-07-03 06:19:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -1351,17 +1351,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>PHYSICAL_PASS_WITH_TEMP_DATA: 両実機で一時URLを使い、削除確認、5秒Undo通知、Undo後の一覧復帰を確認。</t>
+          <t>PASS: Android/iPhone物理実機で削除猶予、Undo通知、対象カード復帰PASS</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>過去試行ではAndroidの座標タップが5秒Undoに間に合わず復元未証明だったが、今回bounds由来のUndo中心タップで復元を確認。iPhoneもAppium/WDA連続操作で復元確認。製品ロジック上の不具合は今回未検出。</t>
+          <t>解消済み: Android Pixel 9aとiPhone 12で削除確認、削除後通知「削除しました」「元に戻す」、Undo後のカード復帰を確認。Supabaseはこの端末内状態遷移の完了条件ではない。</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>2026-07-03 04:45:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>現時点でメモ編集の実機確認上の未解決エラーなし。CoreSimulator/XCTest不整合はこの行の完了判定には使わず、物理実機証跡を正とする。</t>
+          <t>解消済み: Android/iPhone物理実機でメモ編集・保存・詳細反映を確認。Supabaseは端末内メモ編集の完了条件ではない。</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2026-07-03 04:45:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -1886,17 +1886,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_DEVICE_GAP: 両実機で失敗metadataの再取得UI導線と押下を確認。Android/iOSとも再取得・updatedAt不変のRepository契約テストPASS。</t>
+          <t>PARTIAL: local retry contractと両実機の再取得操作は確認、成功metadata更新E2Eは未確認</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>android_device;iphone_device</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-07-03 04:45:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>store_console</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>未完了範囲: iPhone側のタグ管理削除実行、iPhone側の重複タグ名/既割当時文言、iPhone側のタグ別URL件数の物理UI確認。Androidはタグ管理のゴミ箱アイコンのみ表示、一時タグ削除、件数表示、重複/既割当契約を2026-07-03に確認済み。</t>
+          <t>解消済み: Android/iPhone物理実機でタグ作成、同名重複防止、件数表示、ゴミ箱のみの削除UI、削除後の消失を確認。Store consoleはローカルタグ管理の完了条件ではない。</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-07-03 06:50:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>現行コード確認では、ローカル自作タグ詳細は isLocalTag 分岐により「自作タグ」文言、共有タグ専用のクラウドサインイン/共有/参加者表示はSYNCED時だけ表示。過去台帳に残っていたAndroid共有タグ文言混入は現行コードでは再現対象なし。</t>
+          <t>解消済み: 両実機でタグ絞り込み/詳細導線を確認し、現行コードでもLOCAL_ONLY/SYNCED分岐によりローカルタグへ共有タグ専用文言・クラウド操作が混入しない。</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2026-07-03 04:45:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console</t>
+          <t>supabase_auth</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>2026-07-03 07:00:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console;public_web</t>
+          <t>supabase_auth</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2334,17 +2334,17 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>実招待作成/acceptはSupabase liveユーザー状態が必要なため未検証。iPhone実機のinvalid raw error修正後再確認はAppium/usbmuxd復旧待ち。</t>
+          <t>実招待作成/acceptはSupabase liveユーザー状態が必要なため未検証。iPhone実機のinvalid raw error修正後再確認はAppium/usbmuxd復旧待ち。公開invite/reset/privacy/App Links契約は2026-08-13のproduction verifierでPASS。</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>FIXED_LOCAL: Android招待プレビューに12秒タイムアウトを追加し、HTTPS inviteでローディング継続しないようにした。iOSは invalid_or_expired_invite など既知raw errorを日本語文言へ正規化。</t>
+          <t>FIXED_LOCAL_AND_PUBLIC_WEB_VERIFIED: Android招待プレビューに12秒タイムアウトを追加し、iOS既知raw errorを日本語文言へ正規化。Vercel production deployment dpl_52Tc5XaiiLeV9F1EkxTLPXssqRmq の公開invite復帰導線を検証済み。</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest --tests SharedTagAuthViewModelTest --tests ShareReceiverActivityEntrypointTest 成功。PASS: xcodebuild generic iOS Simulator build 成功。PASS Android physical: HTTPS無効招待が「招待リンクが無効か期限切れです」表示へ遷移。iPhone物理再確認はAppium/usbmuxd未復旧のため未実施。</t>
+          <t>PASS local/mobile dated evidence。PASS public 2026-08-13: scripts/verify_public_web_release.shでinvite HTTP 200、コピー/公式Store fallback、reset/privacy/App Links/Universal Links契約を確認。実招待作成・accept・権限同期はSupabase live未検証。</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2359,12 +2359,12 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Deep Link受信/画面遷移は既存の両実機証跡で確認済み。無効リンクUXはAndroid物理PASS、iOSはsource/build修正済み。実際の有効招待作成・参加・権限同期はSupabase liveサインインが必要なためUS-018/US-032側で追跡。</t>
+          <t>公開Webゲートは2026-08-13に解消。実際の有効招待作成・参加・権限同期はSupabase liveサインインが必要なためUS-018/US-032側と合わせて継続追跡。</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2026-07-03 02:59:28 +0900</t>
+          <t>2026-08-13 15:57:37 +0900</t>
         </is>
       </c>
     </row>
@@ -2742,17 +2742,17 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android/iPhone実機でプロフィール編集画面表示PASS、編集保存は未検証</t>
+          <t>PARTIAL: Android/iPhone実機で編集UI表示PASS、プロフィール編集保存は未検証</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>store_console</t>
+          <t>android_device;iphone_device</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>Android/iPhone物理実機でプロフィール名・写真・テーマの編集UIは確認したが、既存ユーザーデータを変更しないため編集保存は未実施。Store consoleはこの未確認操作と無関係。</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>2026-06-29 12:03:48 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console</t>
+          <t>supabase_auth</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>2026-07-03 07:12:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -3170,17 +3170,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android/iPhone実機でエクスポート設定画面PASS、共有シート/ファイル保存実行は未検証</t>
+          <t>PARTIAL: local export testsと両実機の設定画面PASS、物理共有/ファイル保存E2Eは未検証</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>android_device;iphone_device</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>2026-06-29 12:03:48 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>public_web</t>
+          <t>distribution_signing</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Release compile上の失敗なし。署名付き配布や外部console設定はこのストーリーの対象外。</t>
+          <t>Release compileは両OSでPASS。署名付き配布binaryはこのlocal-only検証では作成・実行しておらず、配布署名は別の外部ゲート。</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>2026-07-03 02:54:50 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>PASS_WITH_STORE_GAP: Android/iPhone実機の正準IDとiPhone表示名PASS、ストア表示未検証</t>
+          <t>PASS_WITH_CONFIRMED_APP_STORE_LOCALIZATION_PACKAGING_GAP: 正準ID/公開1.0.17/archive一致PASS、archiveは英語development region・日本語localizationなし</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>store_console</t>
+          <t>distribution_signing;store_console</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3618,17 +3618,17 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>2026-08-13公式App Storeは1.0.17・言語EN。署名済み配布archiveはversion 1.0.17/build 19/canonical bundleとTeam一致、CFBundleDevelopmentRegion=en、CFBundleLocalizationsなし、.lprojなし。current sourceの日本語宣言がarchiveへ反映されていない。</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>SOURCE_DECLARATION_PRESENT / ARCHIVE_NOT_FIXED: current sourceは日本語を宣言するが、公開対応archiveは英語のみ。日本語が実際に含まれる新しい署名archiveを生成・検査してからStore表示を再確認する。</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>PASS exact archive/public boundary 2026-08-13: 公開1.0.17とarchive 1.0.17 (19)/canonical bundle/Teamを照合。archiveはdevelopment region en・localizationなしで、公開EN表示と一致。NOT VERIFIED: corrected archive / App Store Connect post-change localization。</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>実機上の正準Android package/iOS bundle IDは確認済み。App Store/Google Play Console上の表示は未操作。</t>
+          <t>正準ID証拠は維持。App Store EN表示はconsole誤表示ではなく現archiveを正しく反映するため、localization packagingの確認済みMinorとしてdistribution_signing/store_consoleで追跡する。</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>2026-06-29 11:48:00 +0900</t>
+          <t>2026-08-13 17:09:21 +0900</t>
         </is>
       </c>
     </row>
@@ -3832,29 +3832,29 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
+          <t>本番管理者セッションとSupabase Auth/admin権限を使うログイン・非管理者拒否E2Eは未実施。秘密値は表示せず、local build/typecheckのみ確認。</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>修正なし: エラー未検出。</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>再テスト不要: 変更なし。</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>修正なし: エラー未検出。</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>再テスト不要: 変更なし。</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
+      <c r="S32" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="T32" t="inlineStr">
         <is>
           <t>秘密値は扱わない</t>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -3939,37 +3939,37 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
+          <t>本番Supabase管理者セッションでの最新100件一覧・status_label表示E2Eは未実施。local API/source/build検証のみ。</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>修正なし: エラー未検出。</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>再テスト不要: 変更なし。</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>修正なし: エラー未検出。</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>再テスト不要: 変更なし。</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
+      <c r="S33" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
+      <c r="T33" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -4046,29 +4046,29 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
+          <t>本番Supabase管理者セッションとResend live設定を使う優待コード実送信・一度だけの結果確認は未実施。実メール送信はphase 1対象外。</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>修正なし: エラー未検出。</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>再テスト不要: 変更なし。</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>修正なし: エラー未検出。</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>再テスト不要: 変更なし。</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
+      <c r="S34" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="T34" t="inlineStr">
         <is>
           <t>実送信は承認なしにしない</t>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -4153,37 +4153,37 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
+          <t>本番Supabase管理者セッションでの取消POST、revoked_reason永続化、一覧反映E2Eは未実施。</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>修正なし: エラー未検出。</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>再テスト不要: 変更なし。</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>修正なし: エラー未検出。</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>再テスト不要: 変更なし。</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
+      <c r="S35" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
+      <c r="T35" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -4260,37 +4260,37 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
+          <t>本番Supabase Auth管理API権限を使うメール断片検索・非管理者拒否E2Eは未実施。</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>修正なし: エラー未検出。</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>再テスト不要: 変更なし。</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>修正なし: エラー未検出。</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>再テスト不要: 変更なし。</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -4367,37 +4367,37 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
+          <t>本番Resend webhook署名付きイベントとSupabase実DBを使うdelivered/bounced等の反映E2Eは未実施。</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>修正なし: エラー未検出。</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>再テスト不要: 変更なし。</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>修正なし: エラー未検出。</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>再テスト不要: 変更なし。</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -4668,12 +4668,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
+          <t>PASS_LOCAL_BUILD_TEST_WITH_NONBLOCKING_SIMULATOR_WARNING</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>iOS simulator testでCoreSimulator WebCore/WebKit重複クラス警告は残存。物理iPhone UI操作は未検証。</t>
+          <t>非ブロッキング警告: iOS SimulatorのCoreSimulator WebCore/WebKit重複クラス警告は残るが、選択test・署名なしRelease compile・物理iPhone Appium/WDA画面取得はPASS。</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>2026-07-03 07:12:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>supabase_auth;store_console</t>
+          <t>supabase_auth</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>OAuth実ブラウザ往復、Supabase live invite accept、物理iPhone Appium操作は未検証。</t>
+          <t>OAuth実ブラウザ往復、Supabase live invite accept、物理iPhone Appium操作は未検証。公開invite復帰導線は2026-08-13 production verifierでPASS。</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PASS local retest。live invite再開は外部Auth/Supabase環境待ち。 2026-07-03 Android physical: 共有タグ導線からサインイン案内表示PASS。実OAuth/招待リンク再開は未検証。 2026-07-03追加 local/simulator: xcodebuild test -only-testing SharedTagVisibilityTests, SharedTagSyncExecutorTests, URLRulesTests は26 tests PASS。 2026-07-03追加 local: ./gradlew testDebugUnitTest --tests EntitlementResolverTest --tests TagRepositoryTest --tests DetailTagUiStateTest はBUILD SUCCESSFUL。 2026-07-03 07:12追加 iPhone physical via Appium/WDA: PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA): 未ログイン時の共有タグ参加/作成導線としてサインイン案内、メール/パスワード入力欄、サインインボタン要素を確認。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us018-us019-us032-shared-signin-destination.png/xml。実招待リンク保留とサインイン後再開はAuth/Supabase live未検証。</t>
+          <t>PASS local/device dated evidence。PASS public 2026-08-13: scripts/verify_public_web_release.shでinvite HTTP 200とコピー/公式Store fallbackを確認。live invite保留・Auth往復・参加再開は外部Auth/Supabase環境待ち。</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -5141,12 +5141,12 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>実装コミット 7a2aba31。US-017の招待参加から保留再開を分離して追跡。 Android実機で「サインインしていなければ押した時にサインイン案内を出す」挙動は確認済み。 2026-07-03 03:54再確認: CoreDevice/devicectlでは iPhone 12 UDID 00008101-00066D96340A001E が wired/paired/unlocked/tunnel connected。xctraceにもDevices欄で表示。ただし Appium list-real-devices.mjs は usbmuxd 0件、Appium server 127.0.0.1:4723 は未起動、RemoteXPC 42314 は応答なし。root の tunnel-creation PID 71658 はCPU 100%で通常権限kill不可。Appium/WDA操作証跡は継続して NOT VERIFIED on physical iPhone。2026-07-03 04:00再確認: xctraceでは iPhone 12 UDID 00008101-00066D96340A001E が Devices Offline、Appium list-real-devices.mjs は usbmuxd 0件、Appium server 127.0.0.1:4723 は未起動、RemoteXPC 42314 はtimeout。root の tunnel-creation PID 71658 はCPU 100%で通常権限から復旧不可。Appium/WDA操作証跡は継続して NOT VERIFIED on physical iPhone。</t>
+          <t>公開Webゲートは2026-08-13に解消。Android/iOSのpending invite実装は既存証拠どおり。実OAuth/メールサインインとlive invite accept後の再開だけをsupabase_authゲートとして残す。</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>2026-07-03 07:12:00 +0900</t>
+          <t>2026-08-13 15:57:37 +0900</t>
         </is>
       </c>
     </row>
@@ -5524,17 +5524,17 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>FOUNDATION_ONLY_NOT_CANONICAL_UI</t>
+          <t>REMOVED_FROM_CANONICAL_USER_SURFACE_COMPATIBILITY_ONLY</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>public_web;design_required</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>現行正準仕様 docs/rinbam-canonical-spec.md は保存先タグ/自作タグ中心で、コレクション作成・移動UIを採用項目に含めていない。旧台帳ではユーザー機能として残していたため、実機未到達ゲートとして誤追跡していた。</t>
+          <t>解消済み: source-of-truthをdocs/rinbam-canonical-spec.mdへ一本化し、Collection DB/Repositoryは既存データ読込・移行の互換基盤のみ、現行ユーザー機能ではないと明記。再採用は別要件・設計・parity testが必要。</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-07-03 03:00:24 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>supabase_auth;public_web</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -5681,7 +5681,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-07-03 02:52:00 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -5845,17 +5845,17 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>PASS_PUBLIC_WEB_WITH_FINAL_SHA_GAP</t>
+          <t>PUBLIC_WEB_VERIFIED_WITH_STORE_ACCURACY_GATES</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>BLOCKED_EXTERNAL</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>store_console;public_web</t>
+          <t>store_console</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -5865,17 +5865,17 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Play App Signing final SHA-256はNEEDS_USER_ACTION。公開privacy staleは2026-06-29本番deploy後に解消済み。</t>
+          <t>2026-08-13 production verifierはprivacy/account-deletion/reset/invite/assetlinks/AASAを全件PASS。未解決は、cloud-enabled Android v21に対するGoogle Play Data safety不一致、local-only iOS archiveに対するApp Store cloud機能説明不一致、Play App Signing最終SHA-256。Apple privacy Majorはarchive証拠で反証済み。</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>FIXED_PUBLIC_DEPLOY: web/invite-link をVercel project invite-linkへproduction deployし、miyamibu.xyzへalias済み。未修正: final Play SHA-256差し替えはGoogle Play Consoleの外部操作が必要。</t>
+          <t>FIXED_AND_PUBLICLY_VERIFIED: reset/inviteと公開Webは修正・公開済み。Google Data safety MajorとApp Store listing Majorは外部未修正。Apple privacy Majorはmatching local-only archiveによりFALSE_POSITIVE。</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>PASS: npx --yes vercel@latest --prod --yes 成功。deployment dpl_8WZa3BBdqQs4f8s8mKcvxzaspVdv / alias https://miyamibu.xyz。PASS: scripts/verify_public_web_release.sh は privacy/account-deletion HTTP 200、assetlinks/AASA ID、Standard / Pro、Google Play Billing、StoreKit、stale no-real-billing文言なしを全て確認。</t>
+          <t>PASS public 2026-08-13: scripts/verify_public_web_release.sh。BLOCKED_EXTERNAL: Google Data safety修正、App Store product copy/localization修正、Play signing fingerprint照合、post-change公開ページ再確認。</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -5890,12 +5890,12 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>2026-06-29 live privacy staleはproduction deployで解消。残りはPlay Console final SHA-256など外部Console確認のみ。</t>
+          <t>公開Web stale/deployゲートは解消。2026-08-13 C0 read-only Play ConsoleでStep 2 collect/share=yes、Step 5 no collection+shared Web browsing history、account creation does not allow、deletion unansweredを確認。変更/保存は未実施で、Web PASSをStore GOとして扱わない。</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-29 07:25:00 +0900</t>
+          <t>2026-08-13 17:09:21 +0900</t>
         </is>
       </c>
     </row>
@@ -5952,17 +5952,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機で検索欄表示・実データ絞り込みPASS、両OS検索対象unit PASS、iPhone実データ絞り込みは未検証</t>
+          <t>PARTIAL: Android実データ検索と両OSunit/UI操作PASS、iPhone実データ絞り込みE2Eは未検証</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>iphone_device</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-07-03 03:16:04 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_AUTH_MAIL_LIVE_GAP</t>
+          <t>PUBLIC_RESET_PASS_WITH_AUTH_MAIL_LIVE_GAP</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>supabase_auth;public_web</t>
+          <t>supabase_auth</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -6186,17 +6186,17 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Supabase本番メール送信/到達、redirect挙動、物理端末操作は未検証。実メールリンクからのパスワード更新は未検証。</t>
+          <t>Supabase本番メール送信/到達、redirect挙動、実メール recovery code交換とパスワード更新は未検証。公開reset routeのHTTP/CSP契約は2026-08-13 production verifierでPASS。</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>修正なし: US-020から独立した補助機能として台帳追加。</t>
+          <t>PUBLIC_WEB_VERIFIED / AUTH_LIVE_UNVERIFIED: reset routeは外部JS/CSS、厳格CSP、Referrer-Policyと回復契約を実装・公開済み。本番Supabase Auth/SMTPのメール到達は変更も実行もしていない。</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PASS: Android SharedTagAuthViewModelTest継続。PASS Android physical UI: プロフィール/サインイン画面で確認メール再送とパスワード再設定ボタンを確認。live auth mailは外部メール環境待ち。 PASS public web: https://miyamibu.xyz/auth/reset-password はHTTP 200で到達し、パスワード入力/確認、8文字以上、確認一致、updateUser経路の本文を確認。 2026-07-03 07:12追加 iPhone physical via Appium/WDA: PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA): プロフィール/サインイン欄で「確認メール再送」「パスワード再設定」ボタン要素を確認。未入力状態では無効。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-us023-us024-us033-profile-scrolled.png/xml。実メール送信は本番Supabase auth/SMTP live未検証。</t>
+          <t>PASS public 2026-08-13: scripts/verify_public_web_release.shで/auth/reset-password HTTP 200、外部JS/CSS、inline styleなし、CSP契約を確認。PASS既存unit/browser contract。NOT VERIFIED: 本番メール到達・実recovery交換・updateUser。</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -6211,12 +6211,12 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>US-020は基本サインイン系。メール補助は外部メール到達が別ゲート。 targeted unit pass 2026-06-29. reset-password public page source-confirmed 2026-06-29. reset-password public live HTTP 200確認 2026-07-03。 2026-07-03 03:54再確認: CoreDevice/devicectlでは iPhone 12 UDID 00008101-00066D96340A001E が wired/paired/unlocked/tunnel connected。xctraceにもDevices欄で表示。ただし Appium list-real-devices.mjs は usbmuxd 0件、Appium server 127.0.0.1:4723 は未起動、RemoteXPC 42314 は応答なし。root の tunnel-creation PID 71658 はCPU 100%で通常権限kill不可。Appium/WDA操作証跡は継続して NOT VERIFIED on physical iPhone。2026-07-03 04:00再確認: xctraceでは iPhone 12 UDID 00008101-00066D96340A001E が Devices Offline、Appium list-real-devices.mjs は usbmuxd 0件、Appium server 127.0.0.1:4723 は未起動、RemoteXPC 42314 はtimeout。root の tunnel-creation PID 71658 はCPU 100%で通常権限から復旧不可。Appium/WDA操作証跡は継続して NOT VERIFIED on physical iPhone。</t>
+          <t>public_webゲートは解消。残るsupabase_authは実メール送信/到達、redirect、recovery session、更新完了のproduction E2E。秘密値や実アカウントは操作していない。</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-07-03 07:12:00 +0900</t>
+          <t>2026-08-13 15:57:37 +0900</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP: Android/iPhone実機データ取り扱い表示PASS、コード/公開WebローカルPASS、ストア申告未検証</t>
+          <t>PUBLIC_POLICY_VERIFIED_WITH_GOOGLE_DATA_SAFETY_AND_IOS_LISTING_GATES</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>store_console;public_web</t>
+          <t>store_console</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -6293,17 +6293,17 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>物理端末でのAndroidプライバシーダイアログ/iOSデータ取り扱いシート表示とPlay Console/App Store最終申告一致は未検証。修正前のAndroidアプリ内privacy dialogは共有タグクラウド、問い合わせ、Standard/Pro購入を説明していなかった。修正前のiOSはPrivacyInfo.xcprivacyはあったが、アプリ内でユーザーが確認できる同等シートがなかった。live privacy pageの課金なし文言staleは2026-06-29本番deploy後に解消済み。</t>
+          <t>既存実機表示と公開Privacy契約はPASS。署名済みAndroid v21はcloud-enabledなのでGoogle Playのno-data回答と矛盾する。署名済みiOS 1.0.17 (19)はlocal-onlyのためApp Privacy no-dataは矛盾せず、代わりに公開cloud機能説明がbinaryと矛盾する。Consoleは未変更。</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>PARTIAL_FIXED_LOCAL_AND_PUBLIC: Androidアプリ内privacy dialogを、端末内保存、メタデータ取得、共有タグクラウド、問い合わせ送信、Standard/Pro Google Play Billing、広告/分析/クラッシュ収集なしの文言へ更新。iOSはRootViewにinfo.circle入口とPrivacyInfoSheetを追加し、端末内保存、メタデータ取得、共有タグクラウド、問い合わせ、Standard/Pro StoreKit、広告/分析なしを表示。web/invite-link production deployでpublic privacy staleを解消。未修正: store console最終申告一致、物理UI表示確認。</t>
+          <t>PARTIAL_FIXED_LOCAL_AND_PUBLIC / STORE_CONSOLES_UNCHANGED: public Privacyは公開済み。Google Data safety MajorとApp Store listing Majorをdocs化。Play ConsoleはC0がread-only確認、App Store Connectは未操作。Apple privacy Majorは反証済み。</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PASS local: ./gradlew assembleDebug 成功。PASS local: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。PASS local: iOS generic simulator build成功。PASS public: scripts/verify_public_web_release.sh 成功。NOTE: 最初の jp.mimac.urlsaver.AdsConfigTest 指定はテストフィルタ不一致で失敗し、正しい完全修飾名で再実行済み。 2026-07-03再確認: ./scripts/verify_public_web_release.sh PASS。</t>
+          <t>PASS public 2026-08-13: Privacy HTTP 200と既存mobile証拠。BLOCKED_EXTERNAL: Google Data safety修正、App Store listing/localization修正、各post-change public recheck。</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -6318,12 +6318,12 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>Android/iPhoneアプリ内データ取り扱い表示は実機確認済み。Google Play/App Storeのデータセーフティ/広告申告画面は未操作。 2026-07-03時点でも公開privacy/account deletion/AASA/assetlinksはPASS。</t>
+          <t>公開WebはPASS。C0の認証済みPlay Console read-only観測でStep 2/Step 5・account creation・deletion回答の矛盾を確認し、変更/保存は未実施。App Store Connectも未操作。iOS archive反証後もGoogle Major・App Store listing Majorが残りGO不可。</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-07-03 03:36:00 +0900</t>
+          <t>2026-08-13 17:09:21 +0900</t>
         </is>
       </c>
     </row>
@@ -6380,17 +6380,17 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
+          <t>REMOVED_FROM_CANONICAL_USER_SURFACE_COMPATIBILITY_ONLY</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>store_console;public_web;design_required</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>機能基礎はあるが現行ユーザーUI未実装。iOS側にも同等UserLabelモデル/API/UIなし。旧UI復元対象ではなく、公開ユーザー機能にするなら新規仕様判断が必要。</t>
+          <t>解消済み: UserLabel table/column/APIは既存データ・migration互換のため保持するが、現行ユーザー機能ではないと正準仕様へ明記。iOS parityやUIを欠陥として追跡せず、再採用時は別要件とする。</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-06-29 01:49:20 +0900</t>
+          <t>2026-08-11 11:02:17 +0900</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>android_device;distribution_signing;public_privacy;store_console</t>
+          <t>android_device;distribution_signing;store_console</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>未署名AAB・Android物理E2E・iOS Distribution/TestFlight・公開Privacy反映・Store申告は外部ゲート。</t>
+          <t>Android物理E2E・current sourceとのdistribution対応・Google Data safetyは未解決。署名済みAndroid v21 cloud-enabled証拠に対しGoogle no-data回答が矛盾。iOS App Privacy Majorはlocal-only archiveで反証済みだが、App Store cloud機能説明はbinaryと不一致。</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -6838,7 +6838,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>iOS saved-session plus unavailable config now fails closed. Android Release Ads references removed and ChatGPT share intent/cache/25MiB/10000-entry guards added. Redaction now occurs before excerpt clipping with boundary regression tests。未実施: Android物理端末/AVDで直接共有とchooser fallback、Release cold start。iOS最終送信は仕様上実施しない。</t>
+          <t>iOS saved-session plus unavailable config now fails closed. Android Release Ads references removed and ChatGPT share intent/cache/25MiB/10000-entry guards added. Redaction now occurs before excerpt clipping with boundary regression tests。PASS public 2026-08-13: scripts/verify_public_web_release.sh。未実施: Android物理端末/AVDで直接共有とchooser fallback、Release cold start、Store console correction。iOS最終送信は仕様上実施しない。</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -6853,17 +6853,17 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>Chapter 13 is a receiving-side use-case list・not 34 in-app AI features. Canonical fixture: docs/ai/chapter13-chatgpt-use-cases.md.</t>
+          <t>Chapter 13 is a receiving-side use-case list・not 34 in-app AI features. Canonical fixture: docs/ai/chapter13-chatgpt-use-cases.md. public_privacyゲートは解消。Google Data safetyとApp Store listing整合をstore_consoleで継続し、Apple privacy Majorは閉鎖。</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
         <is>
-          <t>2026-07-18 00:00:00 +0900</t>
+          <t>2026-08-13 17:09:21 +0900</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U59"/>
+  <autoFilter ref="A1:U60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6874,7 +6874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6902,220 +6902,174 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>LOCAL_ONLY</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOCAL_ONLY</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>REMOVED</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REMOVED</t>
+          <t>remaining_gate</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>story_ids</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>remaining_gate</t>
+          <t>android_device</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>story_ids</t>
+          <t>US-013,US-021,US-025,CH-013</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>physical_android</t>
+          <t>iphone_device</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t/>
+          <t>US-013,US-021,US-025,US-037</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>physical_iphone</t>
+          <t>distribution_signing</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t/>
+          <t>US-028,US-029,CH-013</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>render_media</t>
+          <t>supabase_auth</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t/>
+          <t>US-016,US-017,US-018,US-019,US-020,US-022,US-023,US-024,AS-001,AS-002,AS-003,AS-004,AS-005,AS-006,ES-005,US-032,US-033,AS-007,AS-008,US-039,AS-009</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>supabase_auth</t>
+          <t>store_console</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-011,US-013,US-015,US-016,US-017,US-018,US-019,US-020,US-022,US-023,US-024,US-025,AS-001,AS-002,AS-003,AS-004,AS-005,AS-006,ES-005,US-032,US-033,AS-007,US-036,AS-008,US-037,US-039,AS-009</t>
+          <t>US-029,US-033,AS-007,ES-006,US-040,CH-013</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>store_console</t>
+          <t>resend_live</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>US-002,US-006,US-014,US-015,US-016,US-017,US-021,US-023,US-029,US-032,US-033,AS-007,ES-006,US-040,TS-001,CH-013</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>resend_live</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
           <t>AS-003,AS-006,AS-008,AS-009</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>public_web</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>US-017,US-028,US-035,US-036,ES-006,US-039,US-040,TS-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>design_required</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>US-035,TS-001</t>
         </is>
       </c>
     </row>

</xml_diff>